<commit_message>
scan: seg6 2026-07-17 18:01 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-17.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-17.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4873,21 +4873,21 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6792</v>
+        <v>6831</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>詠業</t>
+          <t>邁科</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>280.630132591008</v>
+        <v>281.5528979933823</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>53.5</v>
+        <v>612</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>29.26352703858145</v>
+        <v>36.02450233007677</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>19.11649468512422</v>
+        <v>24.17235498332544</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>1.567598666109537</v>
+        <v>0.4754749083376132</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-1.093497252461853</v>
+        <v>-30.43794686603801</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6761</v>
+        <v>6792</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>穩得</t>
+          <t>詠業</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>274.59279588545</v>
+        <v>280.630132591008</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>153</v>
+        <v>53.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>32.01443728555002</v>
+        <v>29.26352703858145</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>16.63657284767011</v>
+        <v>19.11649468512422</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.6646256904027802</v>
+        <v>1.567598666109537</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-3.358256349145637</v>
+        <v>-1.093497252461853</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6671</v>
+        <v>6761</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>三能-KY</t>
+          <t>穩得</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>274.5774052468886</v>
+        <v>274.59279588545</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>24</v>
+        <v>153</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>27.91227646146621</v>
+        <v>32.01443728555002</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>26.84561502432305</v>
+        <v>16.63657284767011</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.7037323293418768</v>
+        <v>0.6646256904027802</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.054634458049073</v>
+        <v>-3.358256349145637</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6788</v>
+        <v>6671</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>三能-KY</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>273.6438923560341</v>
+        <v>274.5774052468886</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>349</v>
+        <v>24</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>32.69315902776925</v>
+        <v>27.91227646146621</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>17.3099294769715</v>
+        <v>26.84561502432305</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.7962026708000656</v>
+        <v>0.7037323293418768</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-7.879633791934101</v>
+        <v>0.054634458049073</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6695</v>
+        <v>6788</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>271.5386245861101</v>
+        <v>273.6438923560341</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>52.3</v>
+        <v>349</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,16 +5110,16 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>43.47100534233831</v>
+        <v>32.69315902776925</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>16.4838830542211</v>
+        <v>17.3099294769715</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.4224613435039707</v>
+        <v>0.7962026708000656</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.7536297305385929</v>
+        <v>-7.879633791934101</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6550</v>
+        <v>6695</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>北極星藥業-KY</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>266.6459105079879</v>
+        <v>271.5386245861101</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>12.2</v>
+        <v>52.3</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>37.29687837207575</v>
+        <v>43.47100534233831</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>20.43294433745979</v>
+        <v>16.4838830542211</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.975252074526582</v>
+        <v>0.4224613435039707</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0086898812394015</v>
+        <v>-0.7536297305385929</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6763</v>
+        <v>6550</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>北極星藥業-KY</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>265.4928559078645</v>
+        <v>266.6459105079879</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>41.8</v>
+        <v>12.2</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>30.4893701955539</v>
+        <v>37.29687837207575</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>20.81459441880098</v>
+        <v>20.43294433745979</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>1.275337220565752</v>
+        <v>0.975252074526582</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.5001521139133187</v>
+        <v>-0.0086898812394015</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6835</v>
+        <v>6763</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>圓裕</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>263.1190895461283</v>
+        <v>265.4928559078645</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>32.05</v>
+        <v>41.8</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>23.3064286768857</v>
+        <v>30.4893701955539</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>34.02737929915874</v>
+        <v>20.81459441880098</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1.444007824254491</v>
+        <v>1.275337220565752</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.2205185810785065</v>
+        <v>-0.5001521139133187</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5297,21 +5297,21 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6560</v>
+        <v>6835</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>欣普羅</t>
+          <t>圓裕</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>259.1748322052993</v>
+        <v>263.1190895461283</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>33</v>
+        <v>32.05</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>26.19112095164185</v>
+        <v>23.3064286768857</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>24.86466235137</v>
+        <v>34.02737929915874</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.8419052993926091</v>
+        <v>1.444007824254491</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.5720345970244697</v>
+        <v>-0.2205185810785065</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5350,21 +5350,21 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6667</v>
+        <v>6560</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>欣普羅</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>258.0260368024004</v>
+        <v>259.1748322052993</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>242</v>
+        <v>33</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>34.61563983640258</v>
+        <v>26.19112095164185</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>13.60574380430473</v>
+        <v>24.86466235137</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.7427082701707092</v>
+        <v>0.8419052993926091</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-2.051481441685209</v>
+        <v>-0.5720345970244697</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6657</v>
+        <v>6667</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>華安</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>252.9920234813595</v>
+        <v>258.0260368024004</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>33.95</v>
+        <v>242</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>41.32586835523217</v>
+        <v>34.61563983640258</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>19.23550351986762</v>
+        <v>13.60574380430473</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>1.937075864911</v>
+        <v>0.7427082701707092</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.027254657737777</v>
+        <v>-2.051481441685209</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6582</v>
+        <v>6657</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>申豐</t>
+          <t>華安</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>252.9518971511319</v>
+        <v>252.9920234813595</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>32.3</v>
+        <v>33.95</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>48.39933465674733</v>
+        <v>41.32586835523217</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>30.71921912654834</v>
+        <v>19.23550351986762</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.5215844390010981</v>
+        <v>1.937075864911</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.1123277405895538</v>
+        <v>-0.027254657737777</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6698</v>
+        <v>6582</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>旭暉應材</t>
+          <t>申豐</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>251.6465976261697</v>
+        <v>252.9518971511319</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>35.6</v>
+        <v>32.3</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>36.67776059611172</v>
+        <v>48.39933465674733</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>21.92670409183246</v>
+        <v>30.71921912654834</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.4291485678141859</v>
+        <v>0.5215844390010981</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.8972672884832709</v>
+        <v>-0.1123277405895538</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6674</v>
+        <v>6698</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>旭暉應材</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>248.3573823601957</v>
+        <v>251.6465976261697</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>15.95</v>
+        <v>35.6</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>36.82600615998278</v>
+        <v>36.67776059611172</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>20.33979880282786</v>
+        <v>21.92670409183246</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>1.526092969433547</v>
+        <v>0.4291485678141859</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.0612364262982789</v>
+        <v>-0.8972672884832709</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6794</v>
+        <v>6674</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>鋐寶科技</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>247.5010677040925</v>
+        <v>248.3573823601957</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>77.40000000000001</v>
+        <v>15.95</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>41.89665491095701</v>
+        <v>36.82600615998278</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>15.90182679211925</v>
+        <v>20.33979880282786</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.941029344679756</v>
+        <v>1.526092969433547</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.2919491172171805</v>
+        <v>-0.0612364262982789</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6592</v>
+        <v>6794</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>和潤企業</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>242.2128276816468</v>
+        <v>247.5010677040925</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>60.4</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>44.22954911306744</v>
+        <v>41.89665491095701</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>21.36279854079797</v>
+        <v>15.90182679211925</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.6230223162571785</v>
+        <v>0.941029344679756</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.083847381035506</v>
+        <v>-0.2919491172171805</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6541</v>
+        <v>6592</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>和潤企業</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>239.1596554169373</v>
+        <v>242.2128276816468</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>38.4</v>
+        <v>60.4</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>40.60413519051495</v>
+        <v>44.22954911306744</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>14.21691791770574</v>
+        <v>21.36279854079797</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>1.113750886540856</v>
+        <v>0.6230223162571785</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.2360789260493613</v>
+        <v>-0.083847381035506</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6781</v>
+        <v>6541</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>233.1913434392887</v>
+        <v>239.1596554169373</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>960</v>
+        <v>38.4</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>31.64067915513114</v>
+        <v>40.60413519051495</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>14.8994328609748</v>
+        <v>14.21691791770574</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>1.079670677249676</v>
+        <v>1.113750886540856</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-22.55149223820933</v>
+        <v>-0.2360789260493613</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6768</v>
+        <v>6781</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>志強-KY</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>232.5832302115936</v>
+        <v>233.1913434392887</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>70</v>
+        <v>960</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>26.64051958716981</v>
+        <v>31.64067915513114</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>32.86622759189652</v>
+        <v>14.8994328609748</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1.390153581108004</v>
+        <v>1.079670677249676</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.226834079241355</v>
+        <v>-22.55149223820933</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6624</v>
+        <v>6768</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>萬年清</t>
+          <t>志強-KY</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>231.3083205123611</v>
+        <v>232.5832302115936</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>44.35</v>
+        <v>70</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>52.62748672911066</v>
+        <v>26.64051958716981</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>7.104105815524484</v>
+        <v>32.86622759189652</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.0444589042205043</v>
+        <v>1.390153581108004</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.6656954700374608</v>
+        <v>-0.226834079241355</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6803</v>
+        <v>6624</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>萬年清</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>229.4601787849016</v>
+        <v>231.3083205123611</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>270</v>
+        <v>44.35</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>26.97254780948199</v>
+        <v>52.62748672911066</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>45.09173357474386</v>
+        <v>7.104105815524484</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1.354243817857163</v>
+        <v>0.0444589042205043</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-1.283031125131823</v>
+        <v>0.6656954700374608</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6689</v>
+        <v>6803</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>227.8397479307405</v>
+        <v>229.4601787849016</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>60.9</v>
+        <v>270</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>35.21469286117507</v>
+        <v>26.97254780948199</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>17.16986272645932</v>
+        <v>45.09173357474386</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>1.511989553931539</v>
+        <v>1.354243817857163</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0641944782130736</v>
+        <v>-1.283031125131823</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6776</v>
+        <v>6689</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>227.4610977898684</v>
+        <v>227.8397479307405</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>53.5</v>
+        <v>60.9</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>36.10582242167144</v>
+        <v>35.21469286117507</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>15.3315636394031</v>
+        <v>17.16986272645932</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1.133293414493478</v>
+        <v>1.511989553931539</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0443016518075498</v>
+        <v>-0.0641944782130736</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6722</v>
+        <v>6776</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>224.5682922525605</v>
+        <v>227.4610977898684</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>33.05</v>
+        <v>53.5</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>31.56738516305731</v>
+        <v>36.10582242167144</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>40.48853622912889</v>
+        <v>15.3315636394031</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.8006493591911176</v>
+        <v>1.133293414493478</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0473856410566158</v>
+        <v>0.0443016518075498</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6546</v>
+        <v>6722</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>210.4700036912417</v>
+        <v>224.5682922525605</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>60.2</v>
+        <v>33.05</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>30.85327967740139</v>
+        <v>31.56738516305731</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>19.01796972680509</v>
+        <v>40.48853622912889</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>1.916544579828935</v>
+        <v>0.8006493591911176</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.8213548300899016</v>
+        <v>-0.0473856410566158</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6591</v>
+        <v>6546</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>209.1757503417756</v>
+        <v>210.4700036912417</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>43.4</v>
+        <v>60.2</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>20.61031309409441</v>
+        <v>30.85327967740139</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>34.49763303844785</v>
+        <v>19.01796972680509</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1.42792599020627</v>
+        <v>1.916544579828935</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.9795732232549256</v>
+        <v>-0.8213548300899016</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6715</v>
+        <v>6591</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>203.9928325496048</v>
+        <v>209.1757503417756</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>391</v>
+        <v>43.4</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>43.5247306421419</v>
+        <v>20.61031309409441</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>13.98154572655759</v>
+        <v>34.49763303844785</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>1.146010854188047</v>
+        <v>1.42792599020627</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-7.772740942127001</v>
+        <v>-0.9795732232549256</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6668</v>
+        <v>6715</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>202.5810939633129</v>
+        <v>203.9928325496048</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>34.6</v>
+        <v>391</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>34.70813685140622</v>
+        <v>43.5247306421419</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.01751541845861</v>
+        <v>13.98154572655759</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.420226077683808</v>
+        <v>1.146010854188047</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.5514903524590191</v>
+        <v>-7.772740942127001</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6605</v>
+        <v>6668</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>198.4228701747622</v>
+        <v>202.5810939633129</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>129</v>
+        <v>34.6</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>40.54468792440669</v>
+        <v>34.70813685140622</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>16.79865209665768</v>
+        <v>17.01751541845861</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.8921049069161318</v>
+        <v>0.420226077683808</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.8236262743263025</v>
+        <v>-0.5514903524590191</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6625</v>
+        <v>6605</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>必應</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>187.1862564164241</v>
+        <v>198.4228701747621</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>77</v>
+        <v>129</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>45.48616799121188</v>
+        <v>40.54468792440669</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>20.49331638779046</v>
+        <v>16.79865209665768</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>1.43188212523811</v>
+        <v>0.8921049069161318</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.3160075985694522</v>
+        <v>-0.8236262743263025</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6692</v>
+        <v>6625</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>必應</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>186.6915197856169</v>
+        <v>187.1862564164241</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>22.75</v>
+        <v>77</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>31.98136711891071</v>
+        <v>45.48616799121188</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>13.19085713247507</v>
+        <v>20.49331638779046</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>2.658587454757769</v>
+        <v>1.43188212523811</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.1175251128899774</v>
+        <v>-0.3160075985694522</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6512</v>
+        <v>6692</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>啟發電</t>
+          <t>進能服</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>184.3112154778575</v>
+        <v>186.6915197856169</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>0</v>
+        <v>22.75</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.57319964816107</v>
+        <v>31.98136711891071</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>11.4893886111829</v>
+        <v>13.19085713247507</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.1688502510101628</v>
+        <v>2.658587454757769</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-1.454940622524211</v>
+        <v>-0.1175251128899774</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6558</v>
+        <v>6512</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>啟發電</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>181.545712540077</v>
+        <v>184.3112154778575</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>27.3</v>
+        <v>0</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>35.29259455000657</v>
+        <v>40.57319964816107</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>16.07211457637777</v>
+        <v>11.4893886111829</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>1.015625048289367</v>
+        <v>0.1688502510101628</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.1510952184038795</v>
+        <v>-1.454940622524211</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6614</v>
+        <v>6558</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>173.9299323879761</v>
+        <v>181.545712540077</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>38.2</v>
+        <v>27.3</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>33.51473993794102</v>
+        <v>35.29259455000657</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>18.23514158205579</v>
+        <v>16.07211457637777</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>1.720064064573152</v>
+        <v>1.015625048289367</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1614917002668286</v>
+        <v>-0.1510952184038795</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6552</v>
+        <v>6614</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>169.23597393918</v>
+        <v>173.9299323879761</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>25.75</v>
+        <v>38.2</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>34.14308243816551</v>
+        <v>33.51473993794102</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>14.33156433801774</v>
+        <v>18.23514158205579</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.9845239736315228</v>
+        <v>1.720064064573152</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.4014845192654422</v>
+        <v>-0.1614917002668286</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6741</v>
+        <v>6552</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>163.719404798172</v>
+        <v>169.23597393918</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>56.7</v>
+        <v>25.75</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>32.50447549107936</v>
+        <v>34.14308243816551</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>19.00716443082947</v>
+        <v>14.33156433801774</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.8919723626065645</v>
+        <v>0.9845239736315228</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.3220728896527045</v>
+        <v>-0.4014845192654422</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6708</v>
+        <v>6741</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>159.1628005474986</v>
+        <v>163.719404798172</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>37.2</v>
+        <v>56.7</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>36.66904198417384</v>
+        <v>32.50447549107936</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>16.31752495492741</v>
+        <v>19.00716443082947</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>1.428465890067951</v>
+        <v>0.8919723626065645</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.1865915026132087</v>
+        <v>-0.3220728896527045</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6504</v>
+        <v>6708</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>南六</t>
+          <t>天擎</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>151.4712728885744</v>
+        <v>159.1628005474986</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>35.8</v>
+        <v>37.2</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>43.86381879550868</v>
+        <v>36.66904198417384</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>13.78442921064745</v>
+        <v>16.31752495492741</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.434196131907943</v>
+        <v>1.428465890067951</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.0908173827968997</v>
+        <v>-0.1865915026132087</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6887,21 +6887,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6597</v>
+        <v>6504</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>南六</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>140.5128924667328</v>
+        <v>151.4712728885744</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>63</v>
+        <v>35.8</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,16 +6912,16 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>49.34138179848882</v>
+        <v>43.86381879550868</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>10.55814476435484</v>
+        <v>13.78442921064745</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.7219931390554073</v>
+        <v>1.434196131907943</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.7370240037144455</v>
+        <v>0.0908173827968997</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6838</v>
+        <v>6597</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>140.0134364672627</v>
+        <v>140.5128924667328</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>22.8</v>
+        <v>63</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>34.13337060590739</v>
+        <v>49.34138179848882</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>10.98228947277887</v>
+        <v>10.55814476435484</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>1.33155152836728</v>
+        <v>0.7219931390554073</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.0267810739872684</v>
+        <v>0.7370240037144455</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6690</v>
+        <v>6838</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>安碁資訊</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>139.6367924489909</v>
+        <v>140.0134364672627</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>159.5</v>
+        <v>22.8</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>35.64512476447148</v>
+        <v>34.13337060590739</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>17.21659709533258</v>
+        <v>10.98228947277887</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>1.26891845342009</v>
+        <v>1.33155152836728</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.3934954532076014</v>
+        <v>-0.0267810739872684</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7046,21 +7046,21 @@
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6796</v>
+        <v>6690</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>晉弘</t>
+          <t>安碁資訊</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>136.2411884783252</v>
+        <v>139.6367924489909</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>57.4</v>
+        <v>159.5</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>43.53463003502061</v>
+        <v>35.64512476447148</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.83492644619994</v>
+        <v>17.21659709533258</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>1.335041724643055</v>
+        <v>1.26891845342009</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.2468277150951198</v>
+        <v>-0.3934954532076014</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7099,21 +7099,21 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6771</v>
+        <v>6796</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>晉弘</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>86.43819053825271</v>
+        <v>136.2411884783252</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>38.5</v>
+        <v>57.4</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,13 +7124,13 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>37.09801935700469</v>
+        <v>43.53463003502061</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>16.70950691778266</v>
+        <v>17.83492644619994</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>1.129776493922357</v>
+        <v>1.335041724643055</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>0</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.0107990534220242</v>
+        <v>0.2468277150951198</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7152,52 +7152,105 @@
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
+        <v>6771</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>平和環保-創</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>86.43819053825271</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>37.09801935700469</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>16.70950691778266</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>1.129776493922357</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
+        <v>0.0107990534220242</v>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
         <v>6720</v>
       </c>
-      <c r="B127" s="2" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>久昌</t>
         </is>
       </c>
-      <c r="C127" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D127" s="2" t="n">
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
         <v>66.26600163792702</v>
       </c>
-      <c r="E127" s="2" t="n">
+      <c r="E128" s="2" t="n">
         <v>138.5</v>
       </c>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="G127" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H127" s="2" t="n">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
         <v>42.64255717066671</v>
       </c>
-      <c r="I127" s="2" t="n">
+      <c r="I128" s="2" t="n">
         <v>19.46794292470927</v>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J128" s="2" t="n">
         <v>0.6625433268674278</v>
       </c>
-      <c r="K127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M127" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N127" s="2" t="n">
+      <c r="K128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
         <v>0.1970667035659632</v>
       </c>
-      <c r="O127" s="2" t="inlineStr">
+      <c r="O128" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>